<commit_message>
order payments and details adjusted
</commit_message>
<xml_diff>
--- a/BOM & CPL/Order-1 by ByteBots.xlsx
+++ b/BOM & CPL/Order-1 by ByteBots.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tawhid\Documents\Github Portfolio\LFR\ByteBot_LFR_V1.0\BOM &amp; CPL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46078057-A038-4902-8D77-A055C9B0DA9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF3E6118-58CA-432D-B42B-1FE8CFE144CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="624" yWindow="2724" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Order-1 by ByteBots" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
   <si>
     <t>Name</t>
   </si>
@@ -99,9 +100,6 @@
     <t>Pololu - Solarbotics RW2i Wheel (internal set screw)</t>
   </si>
   <si>
-    <t>QTRX-MD-07RC Reflectance Sensor Array</t>
-  </si>
-  <si>
     <t>amazon</t>
   </si>
   <si>
@@ -111,9 +109,6 @@
     <t>Pololu Micro Metal Gearmotor Bracket Pair - Black</t>
   </si>
   <si>
-    <t>micro metal gear motor bracket</t>
-  </si>
-  <si>
     <t>motor bracket</t>
   </si>
   <si>
@@ -130,6 +125,15 @@
   </si>
   <si>
     <t>Ship to bd direct</t>
+  </si>
+  <si>
+    <t>micro metal gear motor bracket pair</t>
+  </si>
+  <si>
+    <t>QTR-MD-07RC Reflectance Sensor Array</t>
+  </si>
+  <si>
+    <t>Discount</t>
   </si>
 </sst>
 </file>
@@ -998,19 +1002,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.109375" customWidth="1"/>
     <col min="2" max="2" width="7.6640625" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="3" max="3" width="32" customWidth="1"/>
     <col min="4" max="4" width="23.6640625" customWidth="1"/>
-    <col min="6" max="6" width="19.33203125" customWidth="1"/>
-    <col min="7" max="7" width="63.6640625" customWidth="1"/>
-    <col min="9" max="9" width="14.88671875" customWidth="1"/>
+    <col min="5" max="6" width="15.6640625" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" customWidth="1"/>
+    <col min="8" max="8" width="63.6640625" customWidth="1"/>
+    <col min="10" max="10" width="14.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1027,13 +1032,16 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1047,13 +1055,16 @@
         <v>5</v>
       </c>
       <c r="E2">
-        <v>56</v>
+        <v>59.34</v>
       </c>
       <c r="F2">
-        <v>27.6</v>
+        <v>-9</v>
+      </c>
+      <c r="G2">
+        <v>21.4</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -1064,17 +1075,18 @@
         <v>10</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E3" s="2">
         <v>12</v>
       </c>
       <c r="F3" s="2"/>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2"/>
+      <c r="H3" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -1085,17 +1097,18 @@
         <v>16</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E4" s="2">
         <v>16</v>
       </c>
       <c r="F4" s="2"/>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="2"/>
+      <c r="H4" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -1106,17 +1119,18 @@
         <v>15</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E5" s="2">
         <v>10</v>
       </c>
       <c r="F5" s="2"/>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2"/>
+      <c r="H5" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -1127,20 +1141,20 @@
         <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E6">
-        <f>4.95*2</f>
+        <f>4.95*B6</f>
         <v>9.9</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>24.45</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -1148,80 +1162,88 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="D7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E7">
-        <v>12.42</v>
-      </c>
-      <c r="G7" s="1" t="s">
+        <v>7.24</v>
+      </c>
+      <c r="H7" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B8">
         <v>2</v>
       </c>
       <c r="C8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8">
+        <v>2.95</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>26</v>
-      </c>
-      <c r="D8" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8">
-        <f>2.95*2</f>
-        <v>5.9</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>28</v>
       </c>
       <c r="B9">
         <v>2</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E9">
-        <f>22.45*2</f>
+        <f>22.45*B8</f>
         <v>44.9</v>
       </c>
-      <c r="G9" s="1" t="s">
-        <v>30</v>
+      <c r="H9" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D10" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10">
-        <f>SUM(E2,(E6:E9),(F2:F9))</f>
-        <v>181.17</v>
+        <v>27</v>
+      </c>
+      <c r="E10" t="str">
+        <f>SUM(E2,(E6:E9),(G2:G9),(F2:F9))*121 &amp; " BDT"</f>
+        <v>19502.78 BDT</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G4" r:id="rId1" display="https://www.amazon.com/dp/B0C2Z1WNRV?ref=cm_sw_r_apin_dp_GRAB0R80YQJ3M09K9SNG_2&amp;ref_=cm_sw_r_apin_dp_GRAB0R80YQJ3M09K9SNG_2&amp;social_share=cm_sw_r_apin_dp_GRAB0R80YQJ3M09K9SNG_2&amp;starsLeft=1&amp;th=1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="G3" r:id="rId2" display="https://www.amazon.com/Spektrum-7-4V-300mAh-LiPo-Battery/dp/B0BMFCN7LD/ref=sr_1_55?dib=eyJ2IjoiMSJ9.wzwfGOav2nVI91ccZl7OYcXuXj5Smi1pyHvz8MnEKTZ9i3wTqEBs8eILT9nwq6ENXuUFfiHC3NR4GzKrWZKNDn2YFT1GOJngdxAhUQVP36ZmWMpASlHSShcEF6om4UYc1A77I5Od4scneMemwc5Q7piO5o904nBnSYPnXp5sllmK90l0Z8qhOSYBcrC36MMKfBvg6xPjo1SzN9_ayTyPKAF-JF8dw3SUcm5AlP098XJCQ6lXvSg-kTyhctbc_YtUyZY4NIhVBm0UHuzP0qV-9KIycp-2UfiQ2qPuzQBWwjYV7ewJW2cHAmD6OjKNtzKrRkvC3EkMomIcEg-z-RU6eF-CKgT1zauTDpi5jNGeb0pEI9UUOUbPUmCmcVStcna8lhLiO7oIKxOVe81o1gWduYlHCpAaxtXdjNHLbujBXSE0IcuG8fXP-dL8K9zxNabL.2IexPEltABSEhd3UQSkn-n87hF9K3wfqKcLG_K9WDeA&amp;dib_tag=se&amp;keywords=2s+battery&amp;qid=1740303914&amp;sr=8-55" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="G5" r:id="rId3" display="https://www.amazon.com/dp/B09KM213N7/ref=twister_B09KM3HWH6?_encoding=UTF8&amp;th=1" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="G7" r:id="rId4" location=":~:text=This%20array%20of%20IR%20LED%2Fphototransistor%20pairs%20is%20great,dimmable%20brightness%20control%20independent%20of%20the%20supply%20voltage." display="https://www.pololu.com/product/4147/specs - :~:text=This%20array%20of%20IR%20LED%2Fphototransistor%20pairs%20is%20great,dimmable%20brightness%20control%20independent%20of%20the%20supply%20voltage." xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="G6" r:id="rId5" display="https://www.pololu.com/product/1127" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="G8" r:id="rId6" display="https://www.pololu.com/product/989" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="G9" r:id="rId7" display="https://www.pololu.com/product/3061" xr:uid="{786A8743-C1C8-4FC4-9F17-96B3C408DEC1}"/>
+    <hyperlink ref="H4" r:id="rId1" display="https://www.amazon.com/dp/B0C2Z1WNRV?ref=cm_sw_r_apin_dp_GRAB0R80YQJ3M09K9SNG_2&amp;ref_=cm_sw_r_apin_dp_GRAB0R80YQJ3M09K9SNG_2&amp;social_share=cm_sw_r_apin_dp_GRAB0R80YQJ3M09K9SNG_2&amp;starsLeft=1&amp;th=1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="H3" r:id="rId2" display="https://www.amazon.com/Spektrum-7-4V-300mAh-LiPo-Battery/dp/B0BMFCN7LD/ref=sr_1_55?dib=eyJ2IjoiMSJ9.wzwfGOav2nVI91ccZl7OYcXuXj5Smi1pyHvz8MnEKTZ9i3wTqEBs8eILT9nwq6ENXuUFfiHC3NR4GzKrWZKNDn2YFT1GOJngdxAhUQVP36ZmWMpASlHSShcEF6om4UYc1A77I5Od4scneMemwc5Q7piO5o904nBnSYPnXp5sllmK90l0Z8qhOSYBcrC36MMKfBvg6xPjo1SzN9_ayTyPKAF-JF8dw3SUcm5AlP098XJCQ6lXvSg-kTyhctbc_YtUyZY4NIhVBm0UHuzP0qV-9KIycp-2UfiQ2qPuzQBWwjYV7ewJW2cHAmD6OjKNtzKrRkvC3EkMomIcEg-z-RU6eF-CKgT1zauTDpi5jNGeb0pEI9UUOUbPUmCmcVStcna8lhLiO7oIKxOVe81o1gWduYlHCpAaxtXdjNHLbujBXSE0IcuG8fXP-dL8K9zxNabL.2IexPEltABSEhd3UQSkn-n87hF9K3wfqKcLG_K9WDeA&amp;dib_tag=se&amp;keywords=2s+battery&amp;qid=1740303914&amp;sr=8-55" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="H5" r:id="rId3" display="https://www.amazon.com/dp/B09KM213N7/ref=twister_B09KM3HWH6?_encoding=UTF8&amp;th=1" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="H7" r:id="rId4" location=":~:text=This%20array%20of%20IR%20LED%2Fphototransistor%20pairs%20is%20great,dimmable%20brightness%20control%20independent%20of%20the%20supply%20voltage." display="https://www.pololu.com/product/4147/specs - :~:text=This%20array%20of%20IR%20LED%2Fphototransistor%20pairs%20is%20great,dimmable%20brightness%20control%20independent%20of%20the%20supply%20voltage." xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="H6" r:id="rId5" display="https://www.pololu.com/product/1127" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="H8" r:id="rId6" display="https://www.pololu.com/product/989" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="H9" r:id="rId7" display="https://www.pololu.com/product/3061" xr:uid="{786A8743-C1C8-4FC4-9F17-96B3C408DEC1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId8"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7EE266F-23EE-4292-9755-102F2A0FE031}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>